<commit_message>
fix: universal symmetric plate mirror + annotation angle constraints
weld_extractor:
- Universal pp-mirror: auto-detect symmetric plates by bbox similarity + mirror x
- pp-mirror uses bbox boundary x instead of mirror center for precision
- pp_extra: capture WM arrow positions (3-SIDES + normal WM paths) + view_id
- _redistribute_groups: skip y-offset for different weld pairs at same position
- plate->plate edge x: restrict to edge-on gussets only (_gx_range < 5.0)
- pos-refine: 5mm threshold prevents bad contact edge snaps
- p127: median-y based contact edge selection instead of Counter min

dxf_annotator:
- _redistribute_groups: skip redistribution for different weld pairs
- Angle constraints: reject horizontal (<20deg) AND vertical (>70deg from horiz)
- Pre-filter rejected angles in _search_pass, _fine_tune, _resolve_label_conflicts
</commit_message>
<xml_diff>
--- a/焊缝统计R3_auto(1).xlsx
+++ b/焊缝统计R3_auto(1).xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="17680"/>
+    <workbookView windowHeight="17680"/>
   </bookViews>
   <sheets>
     <sheet name="焊缝统计" sheetId="1" r:id="rId1"/>
@@ -1386,16 +1386,16 @@
     </row>
     <row r="6" hidden="1" spans="1:8">
       <c r="A6" s="4">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="B6" s="4" t="s">
         <v>8</v>
       </c>
       <c r="C6" s="4">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D6" s="4">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>9</v>
@@ -1409,16 +1409,16 @@
     </row>
     <row r="7" hidden="1" spans="1:8">
       <c r="A7" s="4">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B7" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C7" s="4">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="D7" s="4">
-        <v>220</v>
+        <v>300</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>9</v>
@@ -1432,16 +1432,16 @@
     </row>
     <row r="8" hidden="1" spans="1:8">
       <c r="A8" s="4">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>8</v>
       </c>
       <c r="C8" s="4">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D8" s="4">
-        <v>300</v>
+        <v>220</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>9</v>
@@ -1455,16 +1455,16 @@
     </row>
     <row r="9" hidden="1" spans="1:8">
       <c r="A9" s="4">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C9" s="4">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D9" s="4">
-        <v>300</v>
+        <v>220</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>9</v>
@@ -4144,7 +4144,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="126" hidden="1" spans="1:8">
+    <row r="126" spans="1:8">
       <c r="A126" s="4">
         <v>191</v>
       </c>
@@ -4167,7 +4167,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="127" hidden="1" spans="1:8">
+    <row r="127" spans="1:8">
       <c r="A127" s="4">
         <v>192</v>
       </c>
@@ -4190,7 +4190,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="128" hidden="1" spans="1:8">
+    <row r="128" spans="1:8">
       <c r="A128" s="4">
         <v>197</v>
       </c>
@@ -4213,7 +4213,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="129" hidden="1" spans="1:8">
+    <row r="129" spans="1:8">
       <c r="A129" s="4">
         <v>198</v>
       </c>
@@ -4512,7 +4512,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="142" hidden="1" spans="1:8">
+    <row r="142" spans="1:8">
       <c r="A142" s="4">
         <v>187</v>
       </c>
@@ -4535,7 +4535,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="143" ht="12" hidden="1" customHeight="1" spans="1:8">
+    <row r="143" ht="12" customHeight="1" spans="1:8">
       <c r="A143" s="4">
         <v>188</v>
       </c>
@@ -4558,7 +4558,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="144" ht="12" hidden="1" customHeight="1" spans="1:10">
+    <row r="144" ht="12" customHeight="1" spans="1:10">
       <c r="A144" s="4">
         <v>189</v>
       </c>
@@ -4584,7 +4584,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="145" hidden="1" spans="1:8">
+    <row r="145" spans="1:8">
       <c r="A145" s="4">
         <v>190</v>
       </c>
@@ -4607,7 +4607,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="146" hidden="1" spans="1:8">
+    <row r="146" spans="1:8">
       <c r="A146" s="4">
         <v>193</v>
       </c>
@@ -4630,7 +4630,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="147" hidden="1" spans="1:8">
+    <row r="147" spans="1:8">
       <c r="A147" s="4">
         <v>194</v>
       </c>
@@ -4653,7 +4653,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="148" hidden="1" spans="1:8">
+    <row r="148" spans="1:8">
       <c r="A148" s="4">
         <v>195</v>
       </c>
@@ -4676,7 +4676,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="149" hidden="1" spans="1:8">
+    <row r="149" spans="1:8">
       <c r="A149" s="4">
         <v>196</v>
       </c>
@@ -4699,7 +4699,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="150" hidden="1" spans="1:8">
+    <row r="150" spans="1:8">
       <c r="A150" s="4">
         <v>199</v>
       </c>
@@ -4722,7 +4722,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="151" hidden="1" spans="1:8">
+    <row r="151" spans="1:8">
       <c r="A151" s="4">
         <v>200</v>
       </c>
@@ -4929,7 +4929,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="160" hidden="1" spans="1:8">
+    <row r="160" spans="1:8">
       <c r="A160" s="4">
         <v>185</v>
       </c>
@@ -4952,7 +4952,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="161" hidden="1" spans="1:8">
+    <row r="161" spans="1:8">
       <c r="A161" s="4">
         <v>186</v>
       </c>
@@ -4975,7 +4975,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="162" hidden="1" spans="1:8">
+    <row r="162" spans="1:8">
       <c r="A162" s="4">
         <v>207</v>
       </c>
@@ -4998,7 +4998,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="163" hidden="1" spans="1:8">
+    <row r="163" spans="1:8">
       <c r="A163" s="4">
         <v>208</v>
       </c>
@@ -5113,7 +5113,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="168" hidden="1" spans="1:8">
+    <row r="168" spans="1:8">
       <c r="A168" s="4">
         <v>211</v>
       </c>
@@ -5136,7 +5136,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="169" hidden="1" spans="1:8">
+    <row r="169" spans="1:8">
       <c r="A169" s="4">
         <v>212</v>
       </c>
@@ -5159,7 +5159,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="170" hidden="1" spans="1:8">
+    <row r="170" spans="1:8">
       <c r="A170" s="4">
         <v>191</v>
       </c>
@@ -5182,7 +5182,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="171" hidden="1" spans="1:8">
+    <row r="171" spans="1:8">
       <c r="A171" s="4">
         <v>192</v>
       </c>
@@ -5205,7 +5205,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="172" hidden="1" spans="1:8">
+    <row r="172" spans="1:8">
       <c r="A172" s="4">
         <v>197</v>
       </c>
@@ -5228,7 +5228,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="173" hidden="1" spans="1:8">
+    <row r="173" spans="1:8">
       <c r="A173" s="4">
         <v>198</v>
       </c>
@@ -5251,7 +5251,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="174" hidden="1" spans="1:9">
+    <row r="174" spans="1:9">
       <c r="A174" s="4">
         <v>213</v>
       </c>
@@ -5274,7 +5274,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="175" hidden="1" spans="1:9">
+    <row r="175" spans="1:9">
       <c r="A175" s="4">
         <v>217</v>
       </c>
@@ -5343,7 +5343,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="178" ht="12" hidden="1" customHeight="1" spans="1:9">
+    <row r="178" ht="12" customHeight="1" spans="1:9">
       <c r="A178" s="4">
         <v>219</v>
       </c>
@@ -5366,7 +5366,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="179" hidden="1" spans="1:9">
+    <row r="179" spans="1:9">
       <c r="A179" s="4">
         <v>223</v>
       </c>
@@ -5527,7 +5527,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="186" hidden="1" spans="1:8">
+    <row r="186" spans="1:8">
       <c r="A186" s="4">
         <v>203</v>
       </c>
@@ -5550,7 +5550,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="187" hidden="1" spans="1:8">
+    <row r="187" spans="1:8">
       <c r="A187" s="4">
         <v>204</v>
       </c>
@@ -5573,7 +5573,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="188" hidden="1" spans="1:8">
+    <row r="188" spans="1:8">
       <c r="A188" s="4">
         <v>205</v>
       </c>
@@ -5596,7 +5596,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="189" hidden="1" spans="1:8">
+    <row r="189" spans="1:8">
       <c r="A189" s="4">
         <v>206</v>
       </c>
@@ -5619,7 +5619,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="190" hidden="1" spans="1:8">
+    <row r="190" spans="1:8">
       <c r="A190" s="4">
         <v>209</v>
       </c>
@@ -5642,7 +5642,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="191" hidden="1" spans="1:8">
+    <row r="191" spans="1:8">
       <c r="A191" s="4">
         <v>210</v>
       </c>
@@ -5757,7 +5757,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="196" hidden="1" spans="1:9">
+    <row r="196" spans="1:9">
       <c r="A196" s="4">
         <v>215</v>
       </c>
@@ -5780,7 +5780,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="197" hidden="1" spans="1:9">
+    <row r="197" spans="1:9">
       <c r="A197" s="4">
         <v>221</v>
       </c>
@@ -5803,7 +5803,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="198" hidden="1" spans="1:8">
+    <row r="198" spans="1:8">
       <c r="A198" s="4">
         <v>201</v>
       </c>
@@ -5826,7 +5826,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="199" hidden="1" spans="1:8">
+    <row r="199" spans="1:8">
       <c r="A199" s="4">
         <v>202</v>
       </c>
@@ -5849,7 +5849,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="200" hidden="1" spans="1:8">
+    <row r="200" spans="1:8">
       <c r="A200" s="4">
         <v>205</v>
       </c>
@@ -5872,7 +5872,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="201" hidden="1" spans="1:8">
+    <row r="201" spans="1:8">
       <c r="A201" s="4">
         <v>206</v>
       </c>
@@ -5895,7 +5895,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="202" hidden="1" spans="1:8">
+    <row r="202" spans="1:8">
       <c r="A202" s="4">
         <v>183</v>
       </c>
@@ -5918,7 +5918,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="203" ht="10" hidden="1" customHeight="1" spans="1:8">
+    <row r="203" ht="10" customHeight="1" spans="1:8">
       <c r="A203" s="4">
         <v>184</v>
       </c>
@@ -5987,7 +5987,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="206" spans="1:8">
+    <row r="206" hidden="1" spans="1:8">
       <c r="A206" s="4">
         <v>241</v>
       </c>
@@ -6010,7 +6010,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="207" spans="1:8">
+    <row r="207" hidden="1" spans="1:8">
       <c r="A207" s="4">
         <v>242</v>
       </c>
@@ -6033,7 +6033,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="208" spans="1:8">
+    <row r="208" hidden="1" spans="1:8">
       <c r="A208" s="4">
         <v>237</v>
       </c>
@@ -6056,7 +6056,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="209" spans="1:8">
+    <row r="209" hidden="1" spans="1:8">
       <c r="A209" s="4">
         <v>238</v>
       </c>
@@ -6079,7 +6079,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="210" spans="1:8">
+    <row r="210" hidden="1" spans="1:8">
       <c r="A210" s="4">
         <v>239</v>
       </c>
@@ -6102,7 +6102,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="211" spans="1:8">
+    <row r="211" hidden="1" spans="1:8">
       <c r="A211" s="4">
         <v>240</v>
       </c>
@@ -6125,7 +6125,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="212" spans="1:8">
+    <row r="212" hidden="1" spans="1:8">
       <c r="A212" s="4">
         <v>233</v>
       </c>
@@ -6148,7 +6148,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="213" spans="1:8">
+    <row r="213" hidden="1" spans="1:8">
       <c r="A213" s="4">
         <v>234</v>
       </c>
@@ -6171,7 +6171,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="214" spans="1:8">
+    <row r="214" hidden="1" spans="1:8">
       <c r="A214" s="4">
         <v>235</v>
       </c>
@@ -6194,7 +6194,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="215" spans="1:8">
+    <row r="215" hidden="1" spans="1:8">
       <c r="A215" s="4">
         <v>236</v>
       </c>
@@ -6217,7 +6217,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="216" spans="1:8">
+    <row r="216" hidden="1" spans="1:8">
       <c r="A216" s="4">
         <v>247</v>
       </c>
@@ -6240,7 +6240,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="217" spans="1:8">
+    <row r="217" hidden="1" spans="1:8">
       <c r="A217" s="4">
         <v>248</v>
       </c>
@@ -6263,7 +6263,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="218" spans="1:8">
+    <row r="218" hidden="1" spans="1:8">
       <c r="A218" s="4">
         <v>251</v>
       </c>
@@ -6286,7 +6286,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="219" spans="1:8">
+    <row r="219" hidden="1" spans="1:8">
       <c r="A219" s="4">
         <v>252</v>
       </c>
@@ -6309,7 +6309,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="220" spans="1:8">
+    <row r="220" hidden="1" spans="1:8">
       <c r="A220" s="4">
         <v>245</v>
       </c>
@@ -6332,7 +6332,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="221" spans="1:8">
+    <row r="221" hidden="1" spans="1:8">
       <c r="A221" s="4">
         <v>246</v>
       </c>
@@ -6355,7 +6355,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="222" spans="1:8">
+    <row r="222" hidden="1" spans="1:8">
       <c r="A222" s="4">
         <v>249</v>
       </c>
@@ -6378,7 +6378,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="223" spans="1:8">
+    <row r="223" hidden="1" spans="1:8">
       <c r="A223" s="4">
         <v>250</v>
       </c>
@@ -6401,7 +6401,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="224" spans="1:8">
+    <row r="224" hidden="1" spans="1:8">
       <c r="A224" s="4">
         <v>227</v>
       </c>
@@ -6424,7 +6424,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="225" spans="1:8">
+    <row r="225" hidden="1" spans="1:8">
       <c r="A225" s="4">
         <v>228</v>
       </c>
@@ -6447,7 +6447,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="226" spans="1:8">
+    <row r="226" hidden="1" spans="1:8">
       <c r="A226" s="4">
         <v>243</v>
       </c>
@@ -6470,7 +6470,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="227" spans="1:8">
+    <row r="227" hidden="1" spans="1:8">
       <c r="A227" s="4">
         <v>244</v>
       </c>
@@ -6493,7 +6493,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="228" spans="1:8">
+    <row r="228" hidden="1" spans="1:8">
       <c r="A228" s="4">
         <v>231</v>
       </c>
@@ -6516,7 +6516,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="229" spans="1:8">
+    <row r="229" hidden="1" spans="1:8">
       <c r="A229" s="4">
         <v>232</v>
       </c>
@@ -6539,7 +6539,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="230" spans="1:8">
+    <row r="230" hidden="1" spans="1:8">
       <c r="A230" s="4">
         <v>225</v>
       </c>
@@ -6562,7 +6562,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="231" spans="1:8">
+    <row r="231" hidden="1" spans="1:8">
       <c r="A231" s="4">
         <v>226</v>
       </c>
@@ -6585,7 +6585,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="232" spans="1:8">
+    <row r="232" hidden="1" spans="1:8">
       <c r="A232" s="4">
         <v>229</v>
       </c>
@@ -6608,7 +6608,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="233" spans="1:8">
+    <row r="233" hidden="1" spans="1:8">
       <c r="A233" s="4">
         <v>230</v>
       </c>
@@ -10131,11 +10131,11 @@
   <autoFilter xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData" ref="A1:I385" etc:filterBottomFollowUsedRange="0">
     <filterColumn colId="7">
       <filters>
-        <filter val="CO009"/>
+        <filter val="CO008"/>
       </filters>
     </filterColumn>
-    <sortState ref="A1:I385">
-      <sortCondition ref="D1"/>
+    <sortState ref="A2:I385">
+      <sortCondition ref="D1" descending="1"/>
     </sortState>
     <extLst/>
   </autoFilter>

</xml_diff>